<commit_message>
[2D Game Project] 데이터 드리븐 기초
</commit_message>
<xml_diff>
--- a/ExcelFiles/card.xlsx
+++ b/ExcelFiles/card.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\OzProject\UnityBasic_6\JsonConverter\ExcelFiles\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\OzProject\UnityProject\ExcelFiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7DBCCCAC-A53E-4037-81EF-B71E54BEC75E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A229D58-92D1-4E6C-8B86-DEAB52FE9623}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{D0C1FED9-02B4-44E6-A784-5A81E5764927}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="72">
   <si>
     <t>card_punch_01</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -135,52 +135,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>Resources/Image/1</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Resources/Image/2</t>
-  </si>
-  <si>
-    <t>Resources/Image/3</t>
-  </si>
-  <si>
-    <t>Resources/Image/4</t>
-  </si>
-  <si>
-    <t>Resources/Image/5</t>
-  </si>
-  <si>
-    <t>Resources/Image/6</t>
-  </si>
-  <si>
-    <t>Resources/Image/7</t>
-  </si>
-  <si>
-    <t>Resources/Image/8</t>
-  </si>
-  <si>
-    <t>Resources/Image/9</t>
-  </si>
-  <si>
-    <t>Resources/Image/10</t>
-  </si>
-  <si>
-    <t>Resources/Image/11</t>
-  </si>
-  <si>
-    <t>Resources/Image/12</t>
-  </si>
-  <si>
-    <t>Resources/Image/13</t>
-  </si>
-  <si>
-    <t>Resources/Image/14</t>
-  </si>
-  <si>
-    <t>Resources/Image/15</t>
-  </si>
-  <si>
     <t>데미지를 4줍니다</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -253,7 +207,85 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>Address</t>
+    <t>Image/1</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Image/2</t>
+  </si>
+  <si>
+    <t>Image/3</t>
+  </si>
+  <si>
+    <t>Image/4</t>
+  </si>
+  <si>
+    <t>Image/5</t>
+  </si>
+  <si>
+    <t>Image/6</t>
+  </si>
+  <si>
+    <t>Image/7</t>
+  </si>
+  <si>
+    <t>Image/8</t>
+  </si>
+  <si>
+    <t>Image/9</t>
+  </si>
+  <si>
+    <t>Image/10</t>
+  </si>
+  <si>
+    <t>Image/11</t>
+  </si>
+  <si>
+    <t>Image/12</t>
+  </si>
+  <si>
+    <t>Image/13</t>
+  </si>
+  <si>
+    <t>Image/14</t>
+  </si>
+  <si>
+    <t>Image/15</t>
+  </si>
+  <si>
+    <t>ImageIconAddress</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ImageCardAddress</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ImageDamageAddress</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Image/punch_card</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Image/gun_card</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Image/knife_card</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Image/Punch_DamageBackGround</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Image/Gun_DamageBackGround</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Image/Knife_DamageBackGround</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -618,55 +650,63 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{121DAB6B-3E6F-4DF4-85F0-C9EED6886AA7}">
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="27.796875" customWidth="1"/>
     <col min="2" max="2" width="36.5" customWidth="1"/>
     <col min="3" max="4" width="28.5" customWidth="1"/>
     <col min="5" max="5" width="32.796875" customWidth="1"/>
+    <col min="6" max="6" width="28.59765625" customWidth="1"/>
+    <col min="7" max="7" width="22.8984375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A1" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.4">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
-        <v>56</v>
+        <v>41</v>
       </c>
       <c r="B2" t="s">
-        <v>57</v>
+        <v>42</v>
       </c>
       <c r="C2" t="s">
-        <v>58</v>
+        <v>43</v>
       </c>
       <c r="D2" t="s">
-        <v>57</v>
+        <v>42</v>
       </c>
       <c r="E2" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.4">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
-        <v>59</v>
+        <v>44</v>
       </c>
       <c r="B3" t="s">
-        <v>62</v>
+        <v>47</v>
       </c>
       <c r="C3" t="s">
-        <v>61</v>
+        <v>46</v>
       </c>
       <c r="D3" t="s">
-        <v>60</v>
+        <v>45</v>
       </c>
       <c r="E3" t="s">
         <v>63</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="F3" t="s">
+        <v>64</v>
+      </c>
+      <c r="G3" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>0</v>
       </c>
@@ -677,13 +717,19 @@
         <v>4</v>
       </c>
       <c r="D4" t="s">
-        <v>45</v>
+        <v>30</v>
       </c>
       <c r="E4" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.4">
+        <v>48</v>
+      </c>
+      <c r="F4" t="s">
+        <v>66</v>
+      </c>
+      <c r="G4" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>1</v>
       </c>
@@ -694,13 +740,19 @@
         <v>8</v>
       </c>
       <c r="D5" t="s">
-        <v>46</v>
+        <v>31</v>
       </c>
       <c r="E5" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.4">
+        <v>49</v>
+      </c>
+      <c r="F5" t="s">
+        <v>66</v>
+      </c>
+      <c r="G5" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>2</v>
       </c>
@@ -711,13 +763,19 @@
         <v>6</v>
       </c>
       <c r="D6" t="s">
-        <v>47</v>
+        <v>32</v>
       </c>
       <c r="E6" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.4">
+        <v>50</v>
+      </c>
+      <c r="F6" t="s">
+        <v>66</v>
+      </c>
+      <c r="G6" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>3</v>
       </c>
@@ -728,13 +786,19 @@
         <v>2</v>
       </c>
       <c r="D7" t="s">
-        <v>48</v>
+        <v>33</v>
       </c>
       <c r="E7" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.4">
+        <v>51</v>
+      </c>
+      <c r="F7" t="s">
+        <v>66</v>
+      </c>
+      <c r="G7" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
         <v>4</v>
       </c>
@@ -745,13 +809,19 @@
         <v>12</v>
       </c>
       <c r="D8" t="s">
-        <v>49</v>
+        <v>34</v>
       </c>
       <c r="E8" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.4">
+        <v>52</v>
+      </c>
+      <c r="F8" t="s">
+        <v>66</v>
+      </c>
+      <c r="G8" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>5</v>
       </c>
@@ -762,13 +832,19 @@
         <v>4</v>
       </c>
       <c r="D9" t="s">
-        <v>45</v>
+        <v>30</v>
       </c>
       <c r="E9" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.4">
+        <v>53</v>
+      </c>
+      <c r="F9" t="s">
+        <v>67</v>
+      </c>
+      <c r="G9" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
         <v>6</v>
       </c>
@@ -779,13 +855,19 @@
         <v>8</v>
       </c>
       <c r="D10" t="s">
-        <v>46</v>
+        <v>31</v>
       </c>
       <c r="E10" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.4">
+        <v>54</v>
+      </c>
+      <c r="F10" t="s">
+        <v>67</v>
+      </c>
+      <c r="G10" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
         <v>7</v>
       </c>
@@ -796,13 +878,19 @@
         <v>6</v>
       </c>
       <c r="D11" t="s">
-        <v>47</v>
+        <v>32</v>
       </c>
       <c r="E11" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.4">
+        <v>55</v>
+      </c>
+      <c r="F11" t="s">
+        <v>67</v>
+      </c>
+      <c r="G11" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
         <v>8</v>
       </c>
@@ -813,13 +901,19 @@
         <v>2</v>
       </c>
       <c r="D12" t="s">
-        <v>48</v>
+        <v>33</v>
       </c>
       <c r="E12" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.4">
+        <v>56</v>
+      </c>
+      <c r="F12" t="s">
+        <v>67</v>
+      </c>
+      <c r="G12" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
         <v>9</v>
       </c>
@@ -830,13 +924,19 @@
         <v>14</v>
       </c>
       <c r="D13" t="s">
-        <v>50</v>
+        <v>35</v>
       </c>
       <c r="E13" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.4">
+        <v>57</v>
+      </c>
+      <c r="F13" t="s">
+        <v>67</v>
+      </c>
+      <c r="G13" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A14" t="s">
         <v>10</v>
       </c>
@@ -847,13 +947,19 @@
         <v>1</v>
       </c>
       <c r="D14" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="E14" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.4">
+        <v>58</v>
+      </c>
+      <c r="F14" t="s">
+        <v>68</v>
+      </c>
+      <c r="G14" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A15" t="s">
         <v>11</v>
       </c>
@@ -864,13 +970,19 @@
         <v>3</v>
       </c>
       <c r="D15" t="s">
-        <v>52</v>
+        <v>37</v>
       </c>
       <c r="E15" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.4">
+        <v>59</v>
+      </c>
+      <c r="F15" t="s">
+        <v>68</v>
+      </c>
+      <c r="G15" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A16" t="s">
         <v>12</v>
       </c>
@@ -881,13 +993,19 @@
         <v>6</v>
       </c>
       <c r="D16" t="s">
-        <v>47</v>
+        <v>32</v>
       </c>
       <c r="E16" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.4">
+        <v>60</v>
+      </c>
+      <c r="F16" t="s">
+        <v>68</v>
+      </c>
+      <c r="G16" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A17" t="s">
         <v>13</v>
       </c>
@@ -898,13 +1016,19 @@
         <v>9</v>
       </c>
       <c r="D17" t="s">
-        <v>53</v>
+        <v>38</v>
       </c>
       <c r="E17" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.4">
+        <v>61</v>
+      </c>
+      <c r="F17" t="s">
+        <v>68</v>
+      </c>
+      <c r="G17" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A18" t="s">
         <v>14</v>
       </c>
@@ -915,10 +1039,16 @@
         <v>13</v>
       </c>
       <c r="D18" t="s">
-        <v>54</v>
+        <v>39</v>
       </c>
       <c r="E18" t="s">
-        <v>44</v>
+        <v>62</v>
+      </c>
+      <c r="F18" t="s">
+        <v>68</v>
+      </c>
+      <c r="G18" t="s">
+        <v>71</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
[2D Game Project] new card update (ing...)
</commit_message>
<xml_diff>
--- a/ExcelFiles/card.xlsx
+++ b/ExcelFiles/card.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\OzProject\UnityProject\ExcelFiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A229D58-92D1-4E6C-8B86-DEAB52FE9623}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B322F4FB-2CD4-4543-8077-81E1760830F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{D0C1FED9-02B4-44E6-A784-5A81E5764927}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="81">
   <si>
     <t>card_punch_01</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -261,10 +261,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>ImageDamageAddress</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>Image/punch_card</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -277,15 +273,44 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>Image/Punch_DamageBackGround</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Image/Gun_DamageBackGround</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Image/Knife_DamageBackGround</t>
+    <t>card_common_01</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>card_common_02</t>
+  </si>
+  <si>
+    <t>card_common_03</t>
+  </si>
+  <si>
+    <t>card_common_04</t>
+  </si>
+  <si>
+    <t>card_common_05</t>
+  </si>
+  <si>
+    <t>card_common_06</t>
+  </si>
+  <si>
+    <t>card_common_07</t>
+  </si>
+  <si>
+    <t>card_common_08</t>
+  </si>
+  <si>
+    <t>card_common_09</t>
+  </si>
+  <si>
+    <t>card_common_10</t>
+  </si>
+  <si>
+    <t>card_common_11</t>
+  </si>
+  <si>
+    <t>card_common_12</t>
+  </si>
+  <si>
+    <t>Image/common_card</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -650,7 +675,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{121DAB6B-3E6F-4DF4-85F0-C9EED6886AA7}">
-  <dimension ref="A1:G18"/>
+  <dimension ref="A1:F30"/>
   <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="27.796875" customWidth="1"/>
@@ -661,12 +686,12 @@
     <col min="7" max="7" width="22.8984375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A1" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>41</v>
       </c>
@@ -682,8 +707,11 @@
       <c r="E2" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="F2" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>44</v>
       </c>
@@ -702,11 +730,8 @@
       <c r="F3" t="s">
         <v>64</v>
       </c>
-      <c r="G3" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.4">
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>0</v>
       </c>
@@ -723,13 +748,10 @@
         <v>48</v>
       </c>
       <c r="F4" t="s">
-        <v>66</v>
-      </c>
-      <c r="G4" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.4">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>1</v>
       </c>
@@ -746,13 +768,10 @@
         <v>49</v>
       </c>
       <c r="F5" t="s">
-        <v>66</v>
-      </c>
-      <c r="G5" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.4">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>2</v>
       </c>
@@ -769,13 +788,10 @@
         <v>50</v>
       </c>
       <c r="F6" t="s">
-        <v>66</v>
-      </c>
-      <c r="G6" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.4">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>3</v>
       </c>
@@ -792,13 +808,10 @@
         <v>51</v>
       </c>
       <c r="F7" t="s">
-        <v>66</v>
-      </c>
-      <c r="G7" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.4">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
         <v>4</v>
       </c>
@@ -815,13 +828,10 @@
         <v>52</v>
       </c>
       <c r="F8" t="s">
-        <v>66</v>
-      </c>
-      <c r="G8" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.4">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>5</v>
       </c>
@@ -838,13 +848,10 @@
         <v>53</v>
       </c>
       <c r="F9" t="s">
-        <v>67</v>
-      </c>
-      <c r="G9" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.4">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
         <v>6</v>
       </c>
@@ -861,13 +868,10 @@
         <v>54</v>
       </c>
       <c r="F10" t="s">
-        <v>67</v>
-      </c>
-      <c r="G10" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.4">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
         <v>7</v>
       </c>
@@ -884,13 +888,10 @@
         <v>55</v>
       </c>
       <c r="F11" t="s">
-        <v>67</v>
-      </c>
-      <c r="G11" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.4">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
         <v>8</v>
       </c>
@@ -907,13 +908,10 @@
         <v>56</v>
       </c>
       <c r="F12" t="s">
-        <v>67</v>
-      </c>
-      <c r="G12" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.4">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
         <v>9</v>
       </c>
@@ -930,13 +928,10 @@
         <v>57</v>
       </c>
       <c r="F13" t="s">
-        <v>67</v>
-      </c>
-      <c r="G13" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.4">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A14" t="s">
         <v>10</v>
       </c>
@@ -953,13 +948,10 @@
         <v>58</v>
       </c>
       <c r="F14" t="s">
-        <v>68</v>
-      </c>
-      <c r="G14" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.4">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A15" t="s">
         <v>11</v>
       </c>
@@ -976,13 +968,10 @@
         <v>59</v>
       </c>
       <c r="F15" t="s">
-        <v>68</v>
-      </c>
-      <c r="G15" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.4">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A16" t="s">
         <v>12</v>
       </c>
@@ -999,13 +988,10 @@
         <v>60</v>
       </c>
       <c r="F16" t="s">
-        <v>68</v>
-      </c>
-      <c r="G16" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.4">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A17" t="s">
         <v>13</v>
       </c>
@@ -1022,13 +1008,10 @@
         <v>61</v>
       </c>
       <c r="F17" t="s">
-        <v>68</v>
-      </c>
-      <c r="G17" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.4">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A18" t="s">
         <v>14</v>
       </c>
@@ -1045,10 +1028,103 @@
         <v>62</v>
       </c>
       <c r="F18" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A19" t="s">
         <v>68</v>
       </c>
-      <c r="G18" t="s">
+      <c r="F19" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A20" t="s">
+        <v>69</v>
+      </c>
+      <c r="F20" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A21" t="s">
+        <v>70</v>
+      </c>
+      <c r="F21" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A22" t="s">
         <v>71</v>
+      </c>
+      <c r="F22" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A23" t="s">
+        <v>72</v>
+      </c>
+      <c r="F23" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A24" t="s">
+        <v>73</v>
+      </c>
+      <c r="F24" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A25" t="s">
+        <v>74</v>
+      </c>
+      <c r="F25" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A26" t="s">
+        <v>75</v>
+      </c>
+      <c r="F26" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A27" t="s">
+        <v>76</v>
+      </c>
+      <c r="F27" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A28" t="s">
+        <v>77</v>
+      </c>
+      <c r="F28" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A29" t="s">
+        <v>78</v>
+      </c>
+      <c r="F29" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A30" t="s">
+        <v>79</v>
+      </c>
+      <c r="F30" t="s">
+        <v>80</v>
       </c>
     </row>
   </sheetData>

</xml_diff>